<commit_message>
monthly report refactor ui
</commit_message>
<xml_diff>
--- a/public/excelTemplate/import/productTemplate.xlsx
+++ b/public/excelTemplate/import/productTemplate.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9303"/>
   <workbookPr filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="12690" yWindow="-45" windowWidth="16425" windowHeight="12450" activeTab="1"/>
+    <workbookView xWindow="12690" yWindow="-45" windowWidth="16425" windowHeight="12450"/>
   </bookViews>
   <sheets>
     <sheet name="sheet" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="28">
   <si>
     <t>کد کالا</t>
   </si>
@@ -104,6 +104,9 @@
   </si>
   <si>
     <t>شناسه مالیاتی کالا یا خدمت برای ارسال به سامانه مودیان</t>
+  </si>
+  <si>
+    <t>شرح</t>
   </si>
 </sst>
 </file>
@@ -515,7 +518,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -523,7 +526,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" style="2" customWidth="1"/>
@@ -533,11 +536,11 @@
     <col min="6" max="8" width="15.5703125" style="2" customWidth="1"/>
     <col min="9" max="9" width="16.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="22.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.5703125" style="2" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="1"/>
+    <col min="11" max="12" width="17.5703125" style="2" customWidth="1"/>
+    <col min="13" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
@@ -570,6 +573,9 @@
       </c>
       <c r="K1" s="3" t="s">
         <v>25</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>